<commit_message>
add bf-seq column to map-bf-10 results (matches bf 406/500)
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/map-bf/map-bf-10/map-bf-10_schedulables.xlsx
+++ b/workspace/framework_paper/map-bf/map-bf-10/map-bf-10_schedulables.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,11 @@
           <t>bf</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bf-seq</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -478,6 +483,9 @@
       <c r="H2" t="n">
         <v>25</v>
       </c>
+      <c r="I2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -504,6 +512,9 @@
       <c r="H3" t="n">
         <v>25</v>
       </c>
+      <c r="I3" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -530,6 +541,9 @@
       <c r="H4" t="n">
         <v>25</v>
       </c>
+      <c r="I4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -556,6 +570,9 @@
       <c r="H5" t="n">
         <v>25</v>
       </c>
+      <c r="I5" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -582,6 +599,9 @@
       <c r="H6" t="n">
         <v>24</v>
       </c>
+      <c r="I6" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -608,6 +628,9 @@
       <c r="H7" t="n">
         <v>23</v>
       </c>
+      <c r="I7" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -634,6 +657,9 @@
       <c r="H8" t="n">
         <v>22</v>
       </c>
+      <c r="I8" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -660,6 +686,9 @@
       <c r="H9" t="n">
         <v>21</v>
       </c>
+      <c r="I9" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -686,6 +715,9 @@
       <c r="H10" t="n">
         <v>21</v>
       </c>
+      <c r="I10" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -712,6 +744,9 @@
       <c r="H11" t="n">
         <v>21</v>
       </c>
+      <c r="I11" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -738,6 +773,9 @@
       <c r="H12" t="n">
         <v>20</v>
       </c>
+      <c r="I12" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -764,6 +802,9 @@
       <c r="H13" t="n">
         <v>19</v>
       </c>
+      <c r="I13" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -790,6 +831,9 @@
       <c r="H14" t="n">
         <v>19</v>
       </c>
+      <c r="I14" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -816,6 +860,9 @@
       <c r="H15" t="n">
         <v>19</v>
       </c>
+      <c r="I15" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -842,6 +889,9 @@
       <c r="H16" t="n">
         <v>19</v>
       </c>
+      <c r="I16" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -868,6 +918,9 @@
       <c r="H17" t="n">
         <v>18</v>
       </c>
+      <c r="I17" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -894,6 +947,9 @@
       <c r="H18" t="n">
         <v>17</v>
       </c>
+      <c r="I18" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -920,6 +976,9 @@
       <c r="H19" t="n">
         <v>17</v>
       </c>
+      <c r="I19" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -946,6 +1005,9 @@
       <c r="H20" t="n">
         <v>15</v>
       </c>
+      <c r="I20" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -970,6 +1032,9 @@
         <v>10</v>
       </c>
       <c r="H21" t="n">
+        <v>11</v>
+      </c>
+      <c r="I21" t="n">
         <v>11</v>
       </c>
     </row>

</xml_diff>